<commit_message>
Excel mis à jour
</commit_message>
<xml_diff>
--- a/uploads/tableau production baptiste-2-3f599d95.xlsx
+++ b/uploads/tableau production baptiste-2-3f599d95.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baptistedavid/Documents/RECHERCHE TAFF/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baptistedavid/Documents/GitHub/book_social_media/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15160811-83C4-064F-A612-B6BBF58A286F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17A42199-E1EC-7D45-974D-3C16F753B2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,15 +31,15 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Com Radio" guid="{A618CD9D-AFBC-4474-824F-EDA0A02ED83B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Com digitale" guid="{9AD516A6-74B3-445D-BF65-F0FC0B0DC784}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Com corpo" guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtre Com Corpo" guid="{8A52195C-3642-4F94-BF33-9498E684A452}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtre Com Infra" guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtre Team digitale" guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Sanef Solidaire" guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Com Sécurité Routière" guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
     <customWorkbookView name="Filtre Radio" guid="{8594AFCD-3B41-4B81-B979-5456E2FD0AC3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Com Sécurité Routière" guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Sanef Solidaire" guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtre Team digitale" guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtre Com Infra" guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtre Com Corpo" guid="{8A52195C-3642-4F94-BF33-9498E684A452}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Com corpo" guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Com digitale" guid="{9AD516A6-74B3-445D-BF65-F0FC0B0DC784}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Com Radio" guid="{A618CD9D-AFBC-4474-824F-EDA0A02ED83B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -5617,7 +5617,7 @@
         <v>184</v>
       </c>
       <c r="J65" s="20">
-        <v>552200</v>
+        <v>557650</v>
       </c>
       <c r="K65" s="21">
         <v>376544</v>
@@ -6016,7 +6016,7 @@
         <v>200</v>
       </c>
       <c r="J72" s="20">
-        <v>1029677</v>
+        <v>1030026</v>
       </c>
       <c r="K72" s="21">
         <v>628040</v>
@@ -11156,9 +11156,42 @@
     </filterColumn>
   </autoFilter>
   <customSheetViews>
+    <customSheetView guid="{9AD516A6-74B3-445D-BF65-F0FC0B0DC784}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A1:N282" xr:uid="{DAA2786E-BF7D-8D42-A52E-0C3CA22CBB7E}">
+        <filterColumn colId="2">
+          <filters>
+            <filter val="Com digitale"/>
+          </filters>
+        </filterColumn>
+      </autoFilter>
+      <extLst>
+        <ext uri="GoogleSheetsCustomDataVersion1">
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1038187113"/>
+        </ext>
+      </extLst>
+    </customSheetView>
+    <customSheetView guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A1:N282" xr:uid="{4CF23F2B-5439-8945-AF48-599075A0F6BA}"/>
+      <extLst>
+        <ext uri="GoogleSheetsCustomDataVersion1">
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1404300964"/>
+        </ext>
+      </extLst>
+    </customSheetView>
+    <customSheetView guid="{A618CD9D-AFBC-4474-824F-EDA0A02ED83B}" filter="1" showAutoFilter="1">
+      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+      <autoFilter ref="A1:N282" xr:uid="{D84E4817-FCC5-4F4F-9FFA-05167534FB34}"/>
+      <extLst>
+        <ext uri="GoogleSheetsCustomDataVersion1">
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="40062235"/>
+        </ext>
+      </extLst>
+    </customSheetView>
     <customSheetView guid="{E88F7FCD-7F08-4E71-B30C-133DC4379821}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:AB82" xr:uid="{67CB6C46-9DC2-DF44-8363-4E80EABDFB8A}">
+      <autoFilter ref="A1:AB82" xr:uid="{A8368818-79C7-5346-BB71-6D7CA0C0BA0C}">
         <filterColumn colId="3">
           <filters>
             <filter val="LinkedIn"/>
@@ -11168,39 +11201,6 @@
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
           <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="938129022"/>
-        </ext>
-      </extLst>
-    </customSheetView>
-    <customSheetView guid="{A618CD9D-AFBC-4474-824F-EDA0A02ED83B}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N282" xr:uid="{5882B26A-4163-F34B-A4EC-A8E4B8B4EB26}"/>
-      <extLst>
-        <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="40062235"/>
-        </ext>
-      </extLst>
-    </customSheetView>
-    <customSheetView guid="{F190CBEE-8889-45AD-BB7D-398DE1561607}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N282" xr:uid="{741C9B99-BCFD-DB43-92B4-33350D5969D3}"/>
-      <extLst>
-        <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1404300964"/>
-        </ext>
-      </extLst>
-    </customSheetView>
-    <customSheetView guid="{9AD516A6-74B3-445D-BF65-F0FC0B0DC784}" filter="1" showAutoFilter="1">
-      <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N282" xr:uid="{1DFA0880-9244-2545-BE4A-35EC69675E9E}">
-        <filterColumn colId="2">
-          <filters>
-            <filter val="Com digitale"/>
-          </filters>
-        </filterColumn>
-      </autoFilter>
-      <extLst>
-        <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1038187113"/>
         </ext>
       </extLst>
     </customSheetView>
@@ -16420,27 +16420,27 @@
     </filterColumn>
   </autoFilter>
   <customSheetViews>
-    <customSheetView guid="{8A52195C-3642-4F94-BF33-9498E684A452}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{82E21CC6-0589-074C-B3BF-114B203D21D6}"/>
+      <autoFilter ref="A1:N66" xr:uid="{FFF4C445-29CC-E840-90A4-B08AC33E828A}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="270424754"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1311743053"/>
         </ext>
       </extLst>
     </customSheetView>
-    <customSheetView guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{FFF907EB-929C-DE4B-810C-AED92444C459}"/>
+      <autoFilter ref="A1:N230" xr:uid="{6B66FAE9-CFBD-0945-A02B-F2787E274F86}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="213558549"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1754472313"/>
         </ext>
       </extLst>
     </customSheetView>
     <customSheetView guid="{8594AFCD-3B41-4B81-B979-5456E2FD0AC3}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{40E0D96E-0D09-4D44-B697-2DE85F25A5D0}">
+      <autoFilter ref="A1:N66" xr:uid="{D52D9949-BD06-374D-9796-1CAE905C57A9}">
         <filterColumn colId="0">
           <filters blank="1">
             <filter val="December"/>
@@ -16473,21 +16473,21 @@
         </ext>
       </extLst>
     </customSheetView>
-    <customSheetView guid="{6093BE0E-1F80-46F0-B53B-7F4400F2BFE3}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{DB078DD8-52E8-403B-8664-60CFDBD89685}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N230" xr:uid="{EA21761D-817B-3245-9FAC-6BF685DDCA77}"/>
+      <autoFilter ref="A1:N66" xr:uid="{C686C2B3-2811-9545-85FB-3883780BD276}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1754472313"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="213558549"/>
         </ext>
       </extLst>
     </customSheetView>
-    <customSheetView guid="{26B984F1-F5E8-498D-98EF-4918E7E2C674}" filter="1" showAutoFilter="1">
+    <customSheetView guid="{8A52195C-3642-4F94-BF33-9498E684A452}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:N66" xr:uid="{DFB110CA-14D3-834A-8B4C-60749E76DC41}"/>
+      <autoFilter ref="A1:N66" xr:uid="{5F764BAA-745C-354C-AF70-698CA62A0E00}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
-          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="1311743053"/>
+          <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="270424754"/>
         </ext>
       </extLst>
     </customSheetView>

</xml_diff>